<commit_message>
actualizacion de empleados y horarios
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\hikvision-hours-processor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEE07015-02E6-4109-9D53-A7C0543FD843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C2EFDF-1A2F-4F90-B2E5-7B0EE1EADAB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1F8436D6-F06A-412B-A63E-C5B67A15E49B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$29</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="46">
   <si>
     <t>Id</t>
   </si>
@@ -54,9 +57,6 @@
     <t>Mario Butto</t>
   </si>
   <si>
-    <t>Poncio Cristina</t>
-  </si>
-  <si>
     <t>Madera Adrián</t>
   </si>
   <si>
@@ -75,9 +75,6 @@
     <t>Cordoba Gustavo</t>
   </si>
   <si>
-    <t>Flores Rodolfo</t>
-  </si>
-  <si>
     <t>Stieven Emiliano</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>Gimenez Joel</t>
   </si>
   <si>
-    <t>Enriquez Maximiliano</t>
-  </si>
-  <si>
     <t>Moreno Jose Benjamin</t>
   </si>
   <si>
@@ -111,22 +105,13 @@
     <t>Acosta Renzo</t>
   </si>
   <si>
-    <t>Ceballos Facundo</t>
-  </si>
-  <si>
     <t>Borgognoni Tomas</t>
   </si>
   <si>
-    <t>Quiroga Alexis</t>
-  </si>
-  <si>
     <t>Pelliza Roque</t>
   </si>
   <si>
     <t>Gallegos Lucas</t>
-  </si>
-  <si>
-    <t>Funes Leonardo</t>
   </si>
   <si>
     <t>Mansilla Luis Gabriel</t>
@@ -576,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04A9D7D2-8245-49BE-A3DC-DD619418D7D8}">
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I1048570"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" style="1" customWidth="1"/>
@@ -598,25 +583,25 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -639,13 +624,13 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -668,13 +653,13 @@
         <v>0.75</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -697,13 +682,13 @@
         <v>0.75</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -726,49 +711,53 @@
         <v>0.75</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="4">
-        <v>0.34375</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0.5625</v>
+      </c>
       <c r="F6" s="4">
-        <v>0.67638888888888893</v>
+        <v>0.75</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="4">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D7" s="4">
         <v>0.5</v>
@@ -780,24 +769,24 @@
         <v>0.75</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="4">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D8" s="4">
         <v>0.5</v>
@@ -809,97 +798,97 @@
         <v>0.75</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="4">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="D9" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E9" s="4">
-        <v>0.5625</v>
-      </c>
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
       <c r="F9" s="4">
-        <v>0.75</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="4">
-        <v>0.29166666666666669</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="4">
-        <v>0.58333333333333337</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="4">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+        <v>0.3125</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0.5625</v>
+      </c>
       <c r="F11" s="4">
-        <v>0.54166666666666663</v>
+        <v>0.75</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
@@ -917,24 +906,24 @@
         <v>0.75</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="4">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D13" s="4">
         <v>0.5</v>
@@ -946,47 +935,43 @@
         <v>0.75</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="D14" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E14" s="4">
-        <v>0.5625</v>
-      </c>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
       <c r="F14" s="4">
-        <v>0.75</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>15</v>
@@ -1004,43 +989,47 @@
         <v>0.75</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="4">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0.5625</v>
+      </c>
       <c r="F16" s="4">
-        <v>0.58333333333333337</v>
+        <v>0.75</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>17</v>
@@ -1058,82 +1047,74 @@
         <v>0.75</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C18" s="4">
-        <v>0.27083333333333331</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D18" s="4">
         <v>0.5</v>
       </c>
-      <c r="E18" s="4">
-        <v>0.5625</v>
-      </c>
-      <c r="F18" s="4">
-        <v>0.75</v>
-      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
       <c r="G18" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="4">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="D19" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E19" s="4">
-        <v>0.5625</v>
-      </c>
+        <v>0.375</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
       <c r="F19" s="4">
-        <v>0.75</v>
+        <v>0.625</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="4">
-        <v>0.3125</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D20" s="4">
         <v>0.5</v>
@@ -1145,74 +1126,82 @@
         <v>0.75</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C21" s="4">
-        <v>0.33333333333333331</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D21" s="4">
         <v>0.5</v>
       </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
+      <c r="E21" s="4">
+        <v>0.5625</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0.75</v>
+      </c>
       <c r="G21" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C22" s="4">
-        <v>0.375</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+        <v>0.3125</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0.5625</v>
+      </c>
       <c r="F22" s="4">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C23" s="4">
-        <v>0.27083333333333331</v>
+        <v>0.3125</v>
       </c>
       <c r="D23" s="4">
         <v>0.5</v>
@@ -1224,76 +1213,70 @@
         <v>0.75</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="H23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C24" s="4">
-        <v>0.27083333333333331</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D24" s="4">
         <v>0.5</v>
       </c>
-      <c r="E24" s="4">
-        <v>0.5625</v>
-      </c>
-      <c r="F24" s="4">
-        <v>0.75</v>
-      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
       <c r="G24" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C25" s="4">
-        <v>0.33333333333333331</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="D25" s="4">
         <v>0.5</v>
       </c>
       <c r="E25" s="4">
-        <v>0.58333333333333337</v>
+        <v>0.5625</v>
       </c>
       <c r="F25" s="4">
         <v>0.75</v>
       </c>
-      <c r="G25" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="G25" s="2"/>
       <c r="H25" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>26</v>
@@ -1304,83 +1287,73 @@
       <c r="D26" s="4">
         <v>0.5</v>
       </c>
-      <c r="E26" s="4">
-        <v>0.5625</v>
-      </c>
-      <c r="F26" s="4">
-        <v>0.75</v>
-      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C27" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E27" s="4">
-        <v>0.5625</v>
-      </c>
+        <v>0.375</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
       <c r="F27" s="4">
-        <v>0.75</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C28" s="4">
-        <v>0.3125</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="D28" s="4">
         <v>0.5</v>
       </c>
       <c r="E28" s="4">
-        <v>0.5625</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="F28" s="4">
         <v>0.75</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="G28" s="2"/>
       <c r="H28" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>29</v>
@@ -1391,140 +1364,25 @@
       <c r="D29" s="4">
         <v>0.5</v>
       </c>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2" t="s">
-        <v>50</v>
-      </c>
+      <c r="E29" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="F29" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="2">
-        <v>116</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="4">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="D30" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A31" s="2">
-        <v>117</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A32" s="2">
-        <v>118</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A33" s="2">
-        <v>119</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>120</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I34" s="2"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
-        <v>121</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="1048576" spans="7:7" x14ac:dyDescent="0.3">
-      <c r="G1048576" s="2"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="1048570" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G1048570" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I29" xr:uid="{04A9D7D2-8245-49BE-A3DC-DD619418D7D8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>